<commit_message>
chore: aggiorna Template_settimanale.xlsx con colonne K (mese) e L (anno)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/Template_settimanale.xlsx
+++ b/assets/Template_settimanale.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B44DA575-CA51-4FE2-B954-2B121BCDEAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32EAED58-9B8D-B145-90FF-1280CBE4D861}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Monitoraggio finance" sheetId="14" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Monitoraggio finance'!$A$2:$I$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Monitoraggio finance'!$A$1:$L$2</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>MONITORAGGIO FINANCE</t>
   </si>
@@ -59,6 +59,15 @@
   </si>
   <si>
     <t>Includi in PPTX</t>
+  </si>
+  <si>
+    <t>Numero Edizione</t>
+  </si>
+  <si>
+    <t>Mese Edizione</t>
+  </si>
+  <si>
+    <t>Anno Edizione</t>
   </si>
 </sst>
 </file>
@@ -289,7 +298,127 @@
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
     <cellStyle name="Normale 4" xfId="3" xr:uid="{4035A81F-7DCE-4051-9E5B-B9353983DC10}"/>
   </cellStyles>
-  <dxfs count="19">
+  <dxfs count="31">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -782,28 +911,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DD20C8D-D3FC-4EC4-A528-4CD7EE77AC6B}">
-  <dimension ref="A1:I17"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:L17"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.453125" style="4" customWidth="1"/>
-    <col min="2" max="2" width="33.1796875" style="12" customWidth="1"/>
-    <col min="3" max="3" width="25.1796875" style="13" customWidth="1"/>
-    <col min="4" max="5" width="25.1796875" style="4" customWidth="1"/>
-    <col min="6" max="6" width="25.1796875" style="5" customWidth="1"/>
+    <col min="1" max="1" width="10.5" style="4" customWidth="1"/>
+    <col min="2" max="2" width="33.1640625" style="12" customWidth="1"/>
+    <col min="3" max="3" width="25.1640625" style="13" customWidth="1"/>
+    <col min="4" max="5" width="25.1640625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="25.1640625" style="5" customWidth="1"/>
     <col min="7" max="7" width="107" style="6" customWidth="1"/>
-    <col min="8" max="8" width="20.81640625" style="6" customWidth="1"/>
-    <col min="9" max="9" width="76.81640625" style="14" customWidth="1"/>
-    <col min="10" max="16384" width="9.1796875" style="6"/>
+    <col min="8" max="8" width="20.83203125" style="6" customWidth="1"/>
+    <col min="9" max="9" width="76.83203125" style="14" customWidth="1"/>
+    <col min="10" max="10" width="23.1640625" style="6" customWidth="1"/>
+    <col min="11" max="11" width="17.33203125" style="6" customWidth="1"/>
+    <col min="12" max="12" width="16.5" style="6" customWidth="1"/>
+    <col min="13" max="16384" width="9.1640625" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="20.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" ht="20" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="3"/>
     </row>
-    <row r="2" spans="1:9" ht="44.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" ht="44.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="7" t="s">
         <v>1</v>
       </c>
@@ -831,8 +963,17 @@
       <c r="I2" s="11" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" ht="63.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J2" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="K2" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="L2" s="11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="63.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="15"/>
       <c r="B3" s="3"/>
       <c r="C3" s="16"/>
@@ -842,8 +983,11 @@
       <c r="G3" s="19"/>
       <c r="H3" s="16"/>
       <c r="I3" s="1"/>
-    </row>
-    <row r="4" spans="1:9" ht="63.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+    </row>
+    <row r="4" spans="1:12" ht="63.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="15"/>
       <c r="B4" s="3"/>
       <c r="C4" s="16"/>
@@ -853,8 +997,11 @@
       <c r="G4" s="19"/>
       <c r="H4" s="16"/>
       <c r="I4" s="1"/>
-    </row>
-    <row r="5" spans="1:9" ht="63.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+    </row>
+    <row r="5" spans="1:12" ht="63.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="15"/>
       <c r="B5" s="3"/>
       <c r="C5" s="16"/>
@@ -864,8 +1011,11 @@
       <c r="G5" s="19"/>
       <c r="H5" s="16"/>
       <c r="I5" s="1"/>
-    </row>
-    <row r="6" spans="1:9" ht="63.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J5" s="1"/>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+    </row>
+    <row r="6" spans="1:12" ht="63.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="15"/>
       <c r="B6" s="3"/>
       <c r="C6" s="16"/>
@@ -875,8 +1025,11 @@
       <c r="G6" s="19"/>
       <c r="H6" s="16"/>
       <c r="I6" s="1"/>
-    </row>
-    <row r="7" spans="1:9" ht="63.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+    </row>
+    <row r="7" spans="1:12" ht="63.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="15"/>
       <c r="B7" s="3"/>
       <c r="C7" s="16"/>
@@ -886,8 +1039,11 @@
       <c r="G7" s="19"/>
       <c r="H7" s="16"/>
       <c r="I7" s="1"/>
-    </row>
-    <row r="8" spans="1:9" ht="63.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+    </row>
+    <row r="8" spans="1:12" ht="63.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="15"/>
       <c r="B8" s="3"/>
       <c r="C8" s="16"/>
@@ -897,8 +1053,11 @@
       <c r="G8" s="19"/>
       <c r="H8" s="16"/>
       <c r="I8" s="1"/>
-    </row>
-    <row r="9" spans="1:9" ht="63.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+    </row>
+    <row r="9" spans="1:12" ht="63.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="15"/>
       <c r="B9" s="3"/>
       <c r="C9" s="16"/>
@@ -908,8 +1067,11 @@
       <c r="G9" s="19"/>
       <c r="H9" s="16"/>
       <c r="I9" s="1"/>
-    </row>
-    <row r="10" spans="1:9" ht="63.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
+    </row>
+    <row r="10" spans="1:12" ht="63.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="15"/>
       <c r="B10" s="3"/>
       <c r="C10" s="16"/>
@@ -919,8 +1081,11 @@
       <c r="G10" s="19"/>
       <c r="H10" s="16"/>
       <c r="I10" s="1"/>
-    </row>
-    <row r="11" spans="1:9" ht="63.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J10" s="1"/>
+      <c r="K10" s="1"/>
+      <c r="L10" s="1"/>
+    </row>
+    <row r="11" spans="1:12" ht="63.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="15"/>
       <c r="B11" s="3"/>
       <c r="C11" s="16"/>
@@ -930,8 +1095,11 @@
       <c r="G11" s="19"/>
       <c r="H11" s="16"/>
       <c r="I11" s="1"/>
-    </row>
-    <row r="12" spans="1:9" ht="63.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J11" s="1"/>
+      <c r="K11" s="1"/>
+      <c r="L11" s="1"/>
+    </row>
+    <row r="12" spans="1:12" ht="63.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="15"/>
       <c r="B12" s="3"/>
       <c r="C12" s="16"/>
@@ -941,8 +1109,11 @@
       <c r="G12" s="19"/>
       <c r="H12" s="16"/>
       <c r="I12" s="1"/>
-    </row>
-    <row r="13" spans="1:9" ht="63.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J12" s="1"/>
+      <c r="K12" s="1"/>
+      <c r="L12" s="1"/>
+    </row>
+    <row r="13" spans="1:12" ht="63.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="15"/>
       <c r="B13" s="3"/>
       <c r="C13" s="16"/>
@@ -952,8 +1123,11 @@
       <c r="G13" s="19"/>
       <c r="H13" s="16"/>
       <c r="I13" s="1"/>
-    </row>
-    <row r="14" spans="1:9" ht="63.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J13" s="1"/>
+      <c r="K13" s="1"/>
+      <c r="L13" s="1"/>
+    </row>
+    <row r="14" spans="1:12" ht="63.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="15"/>
       <c r="B14" s="3"/>
       <c r="C14" s="16"/>
@@ -963,8 +1137,11 @@
       <c r="G14" s="19"/>
       <c r="H14" s="16"/>
       <c r="I14" s="1"/>
-    </row>
-    <row r="15" spans="1:9" ht="63.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
+      <c r="L14" s="1"/>
+    </row>
+    <row r="15" spans="1:12" ht="63.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="15"/>
       <c r="B15" s="3"/>
       <c r="C15" s="16"/>
@@ -974,8 +1151,11 @@
       <c r="G15" s="19"/>
       <c r="H15" s="16"/>
       <c r="I15" s="1"/>
-    </row>
-    <row r="16" spans="1:9" ht="63.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J15" s="1"/>
+      <c r="K15" s="1"/>
+      <c r="L15" s="1"/>
+    </row>
+    <row r="16" spans="1:12" ht="63.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="15"/>
       <c r="B16" s="3"/>
       <c r="C16" s="16"/>
@@ -985,8 +1165,11 @@
       <c r="G16" s="19"/>
       <c r="H16" s="16"/>
       <c r="I16" s="1"/>
-    </row>
-    <row r="17" spans="1:9" ht="63.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J16" s="1"/>
+      <c r="K16" s="1"/>
+      <c r="L16" s="1"/>
+    </row>
+    <row r="17" spans="1:12" ht="63.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="15"/>
       <c r="B17" s="3"/>
       <c r="C17" s="16"/>
@@ -996,47 +1179,73 @@
       <c r="G17" s="19"/>
       <c r="H17" s="16"/>
       <c r="I17" s="1"/>
+      <c r="J17" s="1"/>
+      <c r="K17" s="1"/>
+      <c r="L17" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:I17" xr:uid="{5DD20C8D-D3FC-4EC4-A528-4CD7EE77AC6B}"/>
   <conditionalFormatting sqref="G1:G1048576">
-    <cfRule type="duplicateValues" dxfId="18" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="G3">
-    <cfRule type="duplicateValues" dxfId="17" priority="768"/>
-    <cfRule type="duplicateValues" dxfId="16" priority="769"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="780"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="781"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="G4">
-    <cfRule type="duplicateValues" dxfId="15" priority="675"/>
-    <cfRule type="duplicateValues" dxfId="14" priority="676"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="687"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="688"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="G5">
-    <cfRule type="duplicateValues" dxfId="13" priority="29"/>
-    <cfRule type="duplicateValues" dxfId="12" priority="30"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="41"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="42"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="G6">
-    <cfRule type="duplicateValues" dxfId="11" priority="770"/>
-    <cfRule type="duplicateValues" dxfId="10" priority="771"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="783"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="782"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="G7:G17">
-    <cfRule type="duplicateValues" dxfId="9" priority="830"/>
-    <cfRule type="duplicateValues" dxfId="8" priority="831"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="843"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="842"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="G18:G1048576 G1">
-    <cfRule type="duplicateValues" dxfId="7" priority="176"/>
-    <cfRule type="duplicateValues" dxfId="6" priority="177"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="188"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="189"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I1:I1048576">
-    <cfRule type="duplicateValues" dxfId="5" priority="8"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="38"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="20"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="50"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I3:I17">
-    <cfRule type="duplicateValues" dxfId="3" priority="840"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="841"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="852"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="853"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I18:I1048576 I1:I2">
-    <cfRule type="duplicateValues" dxfId="1" priority="106"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="108"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="120"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="118"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J2:L2">
+    <cfRule type="duplicateValues" dxfId="11" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="9"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J2:J17">
+    <cfRule type="duplicateValues" dxfId="9" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="7"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J3:J17">
+    <cfRule type="duplicateValues" dxfId="7" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="11"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K2:L2">
+    <cfRule type="duplicateValues" dxfId="4" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K3:L17">
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K3:L17">
+    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="4"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1044,14 +1253,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_Flow_SignoffStatus xmlns="b6280945-9f8f-430a-be42-fa03d44c6387" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -1060,7 +1261,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100A5CA5B64BC909144A63D1E3BABA30816" ma:contentTypeVersion="14" ma:contentTypeDescription="Creare un nuovo documento." ma:contentTypeScope="" ma:versionID="1e1ae5113db714b723ddd659f82498f3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c26730e1-8c85-433e-8fd4-961c6cc6cd52" xmlns:ns3="b6280945-9f8f-430a-be42-fa03d44c6387" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="81dc542ad4b77749a612f076e1db02cd" ns2:_="" ns3:_="">
     <xsd:import namespace="c26730e1-8c85-433e-8fd4-961c6cc6cd52"/>
@@ -1289,24 +1490,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FE64173-066C-4C8C-B58C-03B49B99070E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="b6280945-9f8f-430a-be42-fa03d44c6387"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c26730e1-8c85-433e-8fd4-961c6cc6cd52"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_Flow_SignoffStatus xmlns="b6280945-9f8f-430a-be42-fa03d44c6387" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{202007B8-3D10-446B-AEEE-2A1DD8CFEE5D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -1314,7 +1506,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{39139AFD-824F-4EE1-9C76-329ACFDA2EBA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1331,4 +1523,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1FE64173-066C-4C8C-B58C-03B49B99070E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="b6280945-9f8f-430a-be42-fa03d44c6387"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c26730e1-8c85-433e-8fd4-961c6cc6cd52"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>